<commit_message>
Neue Deals aus Telegram
</commit_message>
<xml_diff>
--- a/deals.xlsx
+++ b/deals.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Deals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -649,23 +649,71 @@
       <c r="N3" s="3" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fertig</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>helly-hansen-womens-verglas-jacket</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Helly Hansen Womens Verglas Jacket</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>119.99</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>49.79</v>
+      </c>
       <c r="F4" s="5">
         <f>IF(AND(ISNUMBER(D4),ISNUMBER(E4),D4&gt;E4),1-E4/D4,"")</f>
         <v/>
       </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="3" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>25.10.2026, 08:59</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Wasserdicht und atmungsaktiv ← optional, kurzer Vorteil fürs Video</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.de/-/en/Helly-Hansen-Womens-Verglas-Jacket/dp/B09Q83R59N/ref=sr_1_6?sr=8-6</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>TOP-DEAL</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>25.10.2026 09:05</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-25_helly-hansen-womens-verglas-jacket.mp4</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="2" t="n"/>

</xml_diff>

<commit_message>
Bot rendert beim Start Zeilen mit Status neu; Hook der Helly-Hansen-Jacke korrigiert
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFAxkANxpPDnbPmm6Aw42Z
</commit_message>
<xml_diff>
--- a/deals.xlsx
+++ b/deals.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Deals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -651,7 +651,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>fertig</t>
+          <t>neu</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Wasserdicht und atmungsaktiv ← optional, kurzer Vorteil fürs Video</t>
+          <t>Wasserdicht und atmungsaktiv</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Neu gerenderte Videos erneut per Telegram senden
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFAxkANxpPDnbPmm6Aw42Z
</commit_message>
<xml_diff>
--- a/deals.xlsx
+++ b/deals.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Deals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -651,7 +651,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>fertig</t>
+          <t>neu</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Tabelle: Spalten Nr und ASIN ergänzt
</commit_message>
<xml_diff>
--- a/deals.xlsx
+++ b/deals.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N201"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -448,6 +448,8 @@
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -521,6 +523,16 @@
           <t>Kategorie</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>ASIN</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -584,6 +596,8 @@
         </is>
       </c>
       <c r="N2" s="3" t="n"/>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -647,6 +661,8 @@
         </is>
       </c>
       <c r="N3" s="3" t="n"/>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="7" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -712,6 +728,14 @@
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Mode</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
+        <is>
+          <t>B09Q83R59N</t>
         </is>
       </c>
     </row>
@@ -733,6 +757,8 @@
       <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="n"/>
       <c r="N5" s="3" t="n"/>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -752,6 +778,8 @@
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="n"/>
       <c r="N6" s="3" t="n"/>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -771,6 +799,8 @@
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="3" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -790,6 +820,8 @@
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="3" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -809,6 +841,8 @@
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="n"/>
       <c r="N9" s="3" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -828,6 +862,8 @@
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7" t="n"/>
       <c r="N10" s="3" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -847,6 +883,8 @@
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="n"/>
       <c r="N11" s="3" t="n"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="n"/>
@@ -866,6 +904,8 @@
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7" t="n"/>
       <c r="N12" s="3" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="n"/>
@@ -885,6 +925,8 @@
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="n"/>
       <c r="N13" s="3" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="n"/>
@@ -904,6 +946,8 @@
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="3" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="2" t="n"/>
@@ -923,6 +967,8 @@
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="n"/>
       <c r="N15" s="3" t="n"/>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="n"/>
@@ -942,6 +988,8 @@
       <c r="L16" s="7" t="n"/>
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="3" t="n"/>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="n"/>
@@ -961,6 +1009,8 @@
       <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="3" t="n"/>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="n"/>
@@ -980,6 +1030,8 @@
       <c r="L18" s="7" t="n"/>
       <c r="M18" s="7" t="n"/>
       <c r="N18" s="3" t="n"/>
+      <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="n"/>
@@ -999,6 +1051,8 @@
       <c r="L19" s="7" t="n"/>
       <c r="M19" s="7" t="n"/>
       <c r="N19" s="3" t="n"/>
+      <c r="O19" s="7" t="n"/>
+      <c r="P19" s="7" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="n"/>
@@ -1018,6 +1072,8 @@
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="3" t="n"/>
+      <c r="O20" s="7" t="n"/>
+      <c r="P20" s="7" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="2" t="n"/>
@@ -1037,6 +1093,8 @@
       <c r="L21" s="7" t="n"/>
       <c r="M21" s="7" t="n"/>
       <c r="N21" s="3" t="n"/>
+      <c r="O21" s="7" t="n"/>
+      <c r="P21" s="7" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="n"/>
@@ -1056,6 +1114,8 @@
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="3" t="n"/>
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="n"/>
@@ -1075,6 +1135,8 @@
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="3" t="n"/>
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="n"/>
@@ -1094,6 +1156,8 @@
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="3" t="n"/>
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="2" t="n"/>
@@ -1113,6 +1177,8 @@
       <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="3" t="n"/>
+      <c r="O25" s="7" t="n"/>
+      <c r="P25" s="7" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="n"/>
@@ -1132,6 +1198,8 @@
       <c r="L26" s="7" t="n"/>
       <c r="M26" s="7" t="n"/>
       <c r="N26" s="3" t="n"/>
+      <c r="O26" s="7" t="n"/>
+      <c r="P26" s="7" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="2" t="n"/>
@@ -1151,6 +1219,8 @@
       <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="n"/>
       <c r="N27" s="3" t="n"/>
+      <c r="O27" s="7" t="n"/>
+      <c r="P27" s="7" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="n"/>
@@ -1170,6 +1240,8 @@
       <c r="L28" s="7" t="n"/>
       <c r="M28" s="7" t="n"/>
       <c r="N28" s="3" t="n"/>
+      <c r="O28" s="7" t="n"/>
+      <c r="P28" s="7" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="2" t="n"/>
@@ -1189,6 +1261,8 @@
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="3" t="n"/>
+      <c r="O29" s="7" t="n"/>
+      <c r="P29" s="7" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2" t="n"/>
@@ -1208,6 +1282,8 @@
       <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="n"/>
       <c r="N30" s="3" t="n"/>
+      <c r="O30" s="7" t="n"/>
+      <c r="P30" s="7" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2" t="n"/>
@@ -1227,6 +1303,8 @@
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
       <c r="N31" s="3" t="n"/>
+      <c r="O31" s="7" t="n"/>
+      <c r="P31" s="7" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2" t="n"/>
@@ -1246,6 +1324,8 @@
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
       <c r="N32" s="3" t="n"/>
+      <c r="O32" s="7" t="n"/>
+      <c r="P32" s="7" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="2" t="n"/>
@@ -1265,6 +1345,8 @@
       <c r="L33" s="7" t="n"/>
       <c r="M33" s="7" t="n"/>
       <c r="N33" s="3" t="n"/>
+      <c r="O33" s="7" t="n"/>
+      <c r="P33" s="7" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2" t="n"/>
@@ -1284,6 +1366,8 @@
       <c r="L34" s="7" t="n"/>
       <c r="M34" s="7" t="n"/>
       <c r="N34" s="3" t="n"/>
+      <c r="O34" s="7" t="n"/>
+      <c r="P34" s="7" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="2" t="n"/>
@@ -1303,6 +1387,8 @@
       <c r="L35" s="7" t="n"/>
       <c r="M35" s="7" t="n"/>
       <c r="N35" s="3" t="n"/>
+      <c r="O35" s="7" t="n"/>
+      <c r="P35" s="7" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="2" t="n"/>
@@ -1322,6 +1408,8 @@
       <c r="L36" s="7" t="n"/>
       <c r="M36" s="7" t="n"/>
       <c r="N36" s="3" t="n"/>
+      <c r="O36" s="7" t="n"/>
+      <c r="P36" s="7" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="2" t="n"/>
@@ -1341,6 +1429,8 @@
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
       <c r="N37" s="3" t="n"/>
+      <c r="O37" s="7" t="n"/>
+      <c r="P37" s="7" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="2" t="n"/>
@@ -1360,6 +1450,8 @@
       <c r="L38" s="7" t="n"/>
       <c r="M38" s="7" t="n"/>
       <c r="N38" s="3" t="n"/>
+      <c r="O38" s="7" t="n"/>
+      <c r="P38" s="7" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="2" t="n"/>
@@ -1379,6 +1471,8 @@
       <c r="L39" s="7" t="n"/>
       <c r="M39" s="7" t="n"/>
       <c r="N39" s="3" t="n"/>
+      <c r="O39" s="7" t="n"/>
+      <c r="P39" s="7" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="2" t="n"/>
@@ -1398,6 +1492,8 @@
       <c r="L40" s="7" t="n"/>
       <c r="M40" s="7" t="n"/>
       <c r="N40" s="3" t="n"/>
+      <c r="O40" s="7" t="n"/>
+      <c r="P40" s="7" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="2" t="n"/>
@@ -1417,6 +1513,8 @@
       <c r="L41" s="7" t="n"/>
       <c r="M41" s="7" t="n"/>
       <c r="N41" s="3" t="n"/>
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="7" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="2" t="n"/>
@@ -1436,6 +1534,8 @@
       <c r="L42" s="7" t="n"/>
       <c r="M42" s="7" t="n"/>
       <c r="N42" s="3" t="n"/>
+      <c r="O42" s="7" t="n"/>
+      <c r="P42" s="7" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="2" t="n"/>
@@ -1455,6 +1555,8 @@
       <c r="L43" s="7" t="n"/>
       <c r="M43" s="7" t="n"/>
       <c r="N43" s="3" t="n"/>
+      <c r="O43" s="7" t="n"/>
+      <c r="P43" s="7" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="2" t="n"/>
@@ -1474,6 +1576,8 @@
       <c r="L44" s="7" t="n"/>
       <c r="M44" s="7" t="n"/>
       <c r="N44" s="3" t="n"/>
+      <c r="O44" s="7" t="n"/>
+      <c r="P44" s="7" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="2" t="n"/>
@@ -1493,6 +1597,8 @@
       <c r="L45" s="7" t="n"/>
       <c r="M45" s="7" t="n"/>
       <c r="N45" s="3" t="n"/>
+      <c r="O45" s="7" t="n"/>
+      <c r="P45" s="7" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="2" t="n"/>
@@ -1512,6 +1618,8 @@
       <c r="L46" s="7" t="n"/>
       <c r="M46" s="7" t="n"/>
       <c r="N46" s="3" t="n"/>
+      <c r="O46" s="7" t="n"/>
+      <c r="P46" s="7" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="2" t="n"/>
@@ -1531,6 +1639,8 @@
       <c r="L47" s="7" t="n"/>
       <c r="M47" s="7" t="n"/>
       <c r="N47" s="3" t="n"/>
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="7" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="2" t="n"/>
@@ -1550,6 +1660,8 @@
       <c r="L48" s="7" t="n"/>
       <c r="M48" s="7" t="n"/>
       <c r="N48" s="3" t="n"/>
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="7" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="2" t="n"/>
@@ -1569,6 +1681,8 @@
       <c r="L49" s="7" t="n"/>
       <c r="M49" s="7" t="n"/>
       <c r="N49" s="3" t="n"/>
+      <c r="O49" s="7" t="n"/>
+      <c r="P49" s="7" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="2" t="n"/>
@@ -1588,6 +1702,8 @@
       <c r="L50" s="7" t="n"/>
       <c r="M50" s="7" t="n"/>
       <c r="N50" s="3" t="n"/>
+      <c r="O50" s="7" t="n"/>
+      <c r="P50" s="7" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="2" t="n"/>
@@ -1607,6 +1723,8 @@
       <c r="L51" s="7" t="n"/>
       <c r="M51" s="7" t="n"/>
       <c r="N51" s="3" t="n"/>
+      <c r="O51" s="7" t="n"/>
+      <c r="P51" s="7" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="2" t="n"/>
@@ -1626,6 +1744,8 @@
       <c r="L52" s="7" t="n"/>
       <c r="M52" s="7" t="n"/>
       <c r="N52" s="3" t="n"/>
+      <c r="O52" s="7" t="n"/>
+      <c r="P52" s="7" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="2" t="n"/>
@@ -1645,6 +1765,8 @@
       <c r="L53" s="7" t="n"/>
       <c r="M53" s="7" t="n"/>
       <c r="N53" s="3" t="n"/>
+      <c r="O53" s="7" t="n"/>
+      <c r="P53" s="7" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="2" t="n"/>
@@ -1664,6 +1786,8 @@
       <c r="L54" s="7" t="n"/>
       <c r="M54" s="7" t="n"/>
       <c r="N54" s="3" t="n"/>
+      <c r="O54" s="7" t="n"/>
+      <c r="P54" s="7" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="2" t="n"/>
@@ -1683,6 +1807,8 @@
       <c r="L55" s="7" t="n"/>
       <c r="M55" s="7" t="n"/>
       <c r="N55" s="3" t="n"/>
+      <c r="O55" s="7" t="n"/>
+      <c r="P55" s="7" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="2" t="n"/>
@@ -1702,6 +1828,8 @@
       <c r="L56" s="7" t="n"/>
       <c r="M56" s="7" t="n"/>
       <c r="N56" s="3" t="n"/>
+      <c r="O56" s="7" t="n"/>
+      <c r="P56" s="7" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="2" t="n"/>
@@ -1721,6 +1849,8 @@
       <c r="L57" s="7" t="n"/>
       <c r="M57" s="7" t="n"/>
       <c r="N57" s="3" t="n"/>
+      <c r="O57" s="7" t="n"/>
+      <c r="P57" s="7" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="2" t="n"/>
@@ -1740,6 +1870,8 @@
       <c r="L58" s="7" t="n"/>
       <c r="M58" s="7" t="n"/>
       <c r="N58" s="3" t="n"/>
+      <c r="O58" s="7" t="n"/>
+      <c r="P58" s="7" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="2" t="n"/>
@@ -1759,6 +1891,8 @@
       <c r="L59" s="7" t="n"/>
       <c r="M59" s="7" t="n"/>
       <c r="N59" s="3" t="n"/>
+      <c r="O59" s="7" t="n"/>
+      <c r="P59" s="7" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="2" t="n"/>
@@ -1778,6 +1912,8 @@
       <c r="L60" s="7" t="n"/>
       <c r="M60" s="7" t="n"/>
       <c r="N60" s="3" t="n"/>
+      <c r="O60" s="7" t="n"/>
+      <c r="P60" s="7" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="2" t="n"/>
@@ -1797,6 +1933,8 @@
       <c r="L61" s="7" t="n"/>
       <c r="M61" s="7" t="n"/>
       <c r="N61" s="3" t="n"/>
+      <c r="O61" s="7" t="n"/>
+      <c r="P61" s="7" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="2" t="n"/>
@@ -1816,6 +1954,8 @@
       <c r="L62" s="7" t="n"/>
       <c r="M62" s="7" t="n"/>
       <c r="N62" s="3" t="n"/>
+      <c r="O62" s="7" t="n"/>
+      <c r="P62" s="7" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="2" t="n"/>
@@ -1835,6 +1975,8 @@
       <c r="L63" s="7" t="n"/>
       <c r="M63" s="7" t="n"/>
       <c r="N63" s="3" t="n"/>
+      <c r="O63" s="7" t="n"/>
+      <c r="P63" s="7" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="2" t="n"/>
@@ -1854,6 +1996,8 @@
       <c r="L64" s="7" t="n"/>
       <c r="M64" s="7" t="n"/>
       <c r="N64" s="3" t="n"/>
+      <c r="O64" s="7" t="n"/>
+      <c r="P64" s="7" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="2" t="n"/>
@@ -1873,6 +2017,8 @@
       <c r="L65" s="7" t="n"/>
       <c r="M65" s="7" t="n"/>
       <c r="N65" s="3" t="n"/>
+      <c r="O65" s="7" t="n"/>
+      <c r="P65" s="7" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="2" t="n"/>
@@ -1892,6 +2038,8 @@
       <c r="L66" s="7" t="n"/>
       <c r="M66" s="7" t="n"/>
       <c r="N66" s="3" t="n"/>
+      <c r="O66" s="7" t="n"/>
+      <c r="P66" s="7" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="2" t="n"/>
@@ -1911,6 +2059,8 @@
       <c r="L67" s="7" t="n"/>
       <c r="M67" s="7" t="n"/>
       <c r="N67" s="3" t="n"/>
+      <c r="O67" s="7" t="n"/>
+      <c r="P67" s="7" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="2" t="n"/>
@@ -1930,6 +2080,8 @@
       <c r="L68" s="7" t="n"/>
       <c r="M68" s="7" t="n"/>
       <c r="N68" s="3" t="n"/>
+      <c r="O68" s="7" t="n"/>
+      <c r="P68" s="7" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="2" t="n"/>
@@ -1949,6 +2101,8 @@
       <c r="L69" s="7" t="n"/>
       <c r="M69" s="7" t="n"/>
       <c r="N69" s="3" t="n"/>
+      <c r="O69" s="7" t="n"/>
+      <c r="P69" s="7" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="2" t="n"/>
@@ -1968,6 +2122,8 @@
       <c r="L70" s="7" t="n"/>
       <c r="M70" s="7" t="n"/>
       <c r="N70" s="3" t="n"/>
+      <c r="O70" s="7" t="n"/>
+      <c r="P70" s="7" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="2" t="n"/>
@@ -1987,6 +2143,8 @@
       <c r="L71" s="7" t="n"/>
       <c r="M71" s="7" t="n"/>
       <c r="N71" s="3" t="n"/>
+      <c r="O71" s="7" t="n"/>
+      <c r="P71" s="7" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="2" t="n"/>
@@ -2006,6 +2164,8 @@
       <c r="L72" s="7" t="n"/>
       <c r="M72" s="7" t="n"/>
       <c r="N72" s="3" t="n"/>
+      <c r="O72" s="7" t="n"/>
+      <c r="P72" s="7" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="2" t="n"/>
@@ -2025,6 +2185,8 @@
       <c r="L73" s="7" t="n"/>
       <c r="M73" s="7" t="n"/>
       <c r="N73" s="3" t="n"/>
+      <c r="O73" s="7" t="n"/>
+      <c r="P73" s="7" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="2" t="n"/>
@@ -2044,6 +2206,8 @@
       <c r="L74" s="7" t="n"/>
       <c r="M74" s="7" t="n"/>
       <c r="N74" s="3" t="n"/>
+      <c r="O74" s="7" t="n"/>
+      <c r="P74" s="7" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="2" t="n"/>
@@ -2063,6 +2227,8 @@
       <c r="L75" s="7" t="n"/>
       <c r="M75" s="7" t="n"/>
       <c r="N75" s="3" t="n"/>
+      <c r="O75" s="7" t="n"/>
+      <c r="P75" s="7" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="2" t="n"/>
@@ -2082,6 +2248,8 @@
       <c r="L76" s="7" t="n"/>
       <c r="M76" s="7" t="n"/>
       <c r="N76" s="3" t="n"/>
+      <c r="O76" s="7" t="n"/>
+      <c r="P76" s="7" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="2" t="n"/>
@@ -2101,6 +2269,8 @@
       <c r="L77" s="7" t="n"/>
       <c r="M77" s="7" t="n"/>
       <c r="N77" s="3" t="n"/>
+      <c r="O77" s="7" t="n"/>
+      <c r="P77" s="7" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="2" t="n"/>
@@ -2120,6 +2290,8 @@
       <c r="L78" s="7" t="n"/>
       <c r="M78" s="7" t="n"/>
       <c r="N78" s="3" t="n"/>
+      <c r="O78" s="7" t="n"/>
+      <c r="P78" s="7" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="2" t="n"/>
@@ -2139,6 +2311,8 @@
       <c r="L79" s="7" t="n"/>
       <c r="M79" s="7" t="n"/>
       <c r="N79" s="3" t="n"/>
+      <c r="O79" s="7" t="n"/>
+      <c r="P79" s="7" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="2" t="n"/>
@@ -2158,6 +2332,8 @@
       <c r="L80" s="7" t="n"/>
       <c r="M80" s="7" t="n"/>
       <c r="N80" s="3" t="n"/>
+      <c r="O80" s="7" t="n"/>
+      <c r="P80" s="7" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="2" t="n"/>
@@ -2177,6 +2353,8 @@
       <c r="L81" s="7" t="n"/>
       <c r="M81" s="7" t="n"/>
       <c r="N81" s="3" t="n"/>
+      <c r="O81" s="7" t="n"/>
+      <c r="P81" s="7" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="2" t="n"/>
@@ -2196,6 +2374,8 @@
       <c r="L82" s="7" t="n"/>
       <c r="M82" s="7" t="n"/>
       <c r="N82" s="3" t="n"/>
+      <c r="O82" s="7" t="n"/>
+      <c r="P82" s="7" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="2" t="n"/>
@@ -2215,6 +2395,8 @@
       <c r="L83" s="7" t="n"/>
       <c r="M83" s="7" t="n"/>
       <c r="N83" s="3" t="n"/>
+      <c r="O83" s="7" t="n"/>
+      <c r="P83" s="7" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="2" t="n"/>
@@ -2234,6 +2416,8 @@
       <c r="L84" s="7" t="n"/>
       <c r="M84" s="7" t="n"/>
       <c r="N84" s="3" t="n"/>
+      <c r="O84" s="7" t="n"/>
+      <c r="P84" s="7" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="2" t="n"/>
@@ -2253,6 +2437,8 @@
       <c r="L85" s="7" t="n"/>
       <c r="M85" s="7" t="n"/>
       <c r="N85" s="3" t="n"/>
+      <c r="O85" s="7" t="n"/>
+      <c r="P85" s="7" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="2" t="n"/>
@@ -2272,6 +2458,8 @@
       <c r="L86" s="7" t="n"/>
       <c r="M86" s="7" t="n"/>
       <c r="N86" s="3" t="n"/>
+      <c r="O86" s="7" t="n"/>
+      <c r="P86" s="7" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="2" t="n"/>
@@ -2291,6 +2479,8 @@
       <c r="L87" s="7" t="n"/>
       <c r="M87" s="7" t="n"/>
       <c r="N87" s="3" t="n"/>
+      <c r="O87" s="7" t="n"/>
+      <c r="P87" s="7" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="2" t="n"/>
@@ -2310,6 +2500,8 @@
       <c r="L88" s="7" t="n"/>
       <c r="M88" s="7" t="n"/>
       <c r="N88" s="3" t="n"/>
+      <c r="O88" s="7" t="n"/>
+      <c r="P88" s="7" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="2" t="n"/>
@@ -2329,6 +2521,8 @@
       <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="n"/>
       <c r="N89" s="3" t="n"/>
+      <c r="O89" s="7" t="n"/>
+      <c r="P89" s="7" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="2" t="n"/>
@@ -2348,6 +2542,8 @@
       <c r="L90" s="7" t="n"/>
       <c r="M90" s="7" t="n"/>
       <c r="N90" s="3" t="n"/>
+      <c r="O90" s="7" t="n"/>
+      <c r="P90" s="7" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="2" t="n"/>
@@ -2367,6 +2563,8 @@
       <c r="L91" s="7" t="n"/>
       <c r="M91" s="7" t="n"/>
       <c r="N91" s="3" t="n"/>
+      <c r="O91" s="7" t="n"/>
+      <c r="P91" s="7" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="2" t="n"/>
@@ -2386,6 +2584,8 @@
       <c r="L92" s="7" t="n"/>
       <c r="M92" s="7" t="n"/>
       <c r="N92" s="3" t="n"/>
+      <c r="O92" s="7" t="n"/>
+      <c r="P92" s="7" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="2" t="n"/>
@@ -2405,6 +2605,8 @@
       <c r="L93" s="7" t="n"/>
       <c r="M93" s="7" t="n"/>
       <c r="N93" s="3" t="n"/>
+      <c r="O93" s="7" t="n"/>
+      <c r="P93" s="7" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="2" t="n"/>
@@ -2424,6 +2626,8 @@
       <c r="L94" s="7" t="n"/>
       <c r="M94" s="7" t="n"/>
       <c r="N94" s="3" t="n"/>
+      <c r="O94" s="7" t="n"/>
+      <c r="P94" s="7" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="2" t="n"/>
@@ -2443,6 +2647,8 @@
       <c r="L95" s="7" t="n"/>
       <c r="M95" s="7" t="n"/>
       <c r="N95" s="3" t="n"/>
+      <c r="O95" s="7" t="n"/>
+      <c r="P95" s="7" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="2" t="n"/>
@@ -2462,6 +2668,8 @@
       <c r="L96" s="7" t="n"/>
       <c r="M96" s="7" t="n"/>
       <c r="N96" s="3" t="n"/>
+      <c r="O96" s="7" t="n"/>
+      <c r="P96" s="7" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="2" t="n"/>
@@ -2481,6 +2689,8 @@
       <c r="L97" s="7" t="n"/>
       <c r="M97" s="7" t="n"/>
       <c r="N97" s="3" t="n"/>
+      <c r="O97" s="7" t="n"/>
+      <c r="P97" s="7" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="2" t="n"/>
@@ -2500,6 +2710,8 @@
       <c r="L98" s="7" t="n"/>
       <c r="M98" s="7" t="n"/>
       <c r="N98" s="3" t="n"/>
+      <c r="O98" s="7" t="n"/>
+      <c r="P98" s="7" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="2" t="n"/>
@@ -2519,6 +2731,8 @@
       <c r="L99" s="7" t="n"/>
       <c r="M99" s="7" t="n"/>
       <c r="N99" s="3" t="n"/>
+      <c r="O99" s="7" t="n"/>
+      <c r="P99" s="7" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="2" t="n"/>
@@ -2538,6 +2752,8 @@
       <c r="L100" s="7" t="n"/>
       <c r="M100" s="7" t="n"/>
       <c r="N100" s="3" t="n"/>
+      <c r="O100" s="7" t="n"/>
+      <c r="P100" s="7" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="2" t="n"/>
@@ -2557,6 +2773,8 @@
       <c r="L101" s="7" t="n"/>
       <c r="M101" s="7" t="n"/>
       <c r="N101" s="3" t="n"/>
+      <c r="O101" s="7" t="n"/>
+      <c r="P101" s="7" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="2" t="n"/>
@@ -2576,6 +2794,8 @@
       <c r="L102" s="7" t="n"/>
       <c r="M102" s="7" t="n"/>
       <c r="N102" s="3" t="n"/>
+      <c r="O102" s="7" t="n"/>
+      <c r="P102" s="7" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="2" t="n"/>
@@ -2595,6 +2815,8 @@
       <c r="L103" s="7" t="n"/>
       <c r="M103" s="7" t="n"/>
       <c r="N103" s="3" t="n"/>
+      <c r="O103" s="7" t="n"/>
+      <c r="P103" s="7" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1">
       <c r="A104" s="2" t="n"/>
@@ -2614,6 +2836,8 @@
       <c r="L104" s="7" t="n"/>
       <c r="M104" s="7" t="n"/>
       <c r="N104" s="3" t="n"/>
+      <c r="O104" s="7" t="n"/>
+      <c r="P104" s="7" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1">
       <c r="A105" s="2" t="n"/>
@@ -2633,6 +2857,8 @@
       <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="n"/>
       <c r="N105" s="3" t="n"/>
+      <c r="O105" s="7" t="n"/>
+      <c r="P105" s="7" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" s="2" t="n"/>
@@ -2652,6 +2878,8 @@
       <c r="L106" s="7" t="n"/>
       <c r="M106" s="7" t="n"/>
       <c r="N106" s="3" t="n"/>
+      <c r="O106" s="7" t="n"/>
+      <c r="P106" s="7" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" s="2" t="n"/>
@@ -2671,6 +2899,8 @@
       <c r="L107" s="7" t="n"/>
       <c r="M107" s="7" t="n"/>
       <c r="N107" s="3" t="n"/>
+      <c r="O107" s="7" t="n"/>
+      <c r="P107" s="7" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1">
       <c r="A108" s="2" t="n"/>
@@ -2690,6 +2920,8 @@
       <c r="L108" s="7" t="n"/>
       <c r="M108" s="7" t="n"/>
       <c r="N108" s="3" t="n"/>
+      <c r="O108" s="7" t="n"/>
+      <c r="P108" s="7" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="2" t="n"/>
@@ -2709,6 +2941,8 @@
       <c r="L109" s="7" t="n"/>
       <c r="M109" s="7" t="n"/>
       <c r="N109" s="3" t="n"/>
+      <c r="O109" s="7" t="n"/>
+      <c r="P109" s="7" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="A110" s="2" t="n"/>
@@ -2728,6 +2962,8 @@
       <c r="L110" s="7" t="n"/>
       <c r="M110" s="7" t="n"/>
       <c r="N110" s="3" t="n"/>
+      <c r="O110" s="7" t="n"/>
+      <c r="P110" s="7" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1">
       <c r="A111" s="2" t="n"/>
@@ -2747,6 +2983,8 @@
       <c r="L111" s="7" t="n"/>
       <c r="M111" s="7" t="n"/>
       <c r="N111" s="3" t="n"/>
+      <c r="O111" s="7" t="n"/>
+      <c r="P111" s="7" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1">
       <c r="A112" s="2" t="n"/>
@@ -2766,6 +3004,8 @@
       <c r="L112" s="7" t="n"/>
       <c r="M112" s="7" t="n"/>
       <c r="N112" s="3" t="n"/>
+      <c r="O112" s="7" t="n"/>
+      <c r="P112" s="7" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1">
       <c r="A113" s="2" t="n"/>
@@ -2785,6 +3025,8 @@
       <c r="L113" s="7" t="n"/>
       <c r="M113" s="7" t="n"/>
       <c r="N113" s="3" t="n"/>
+      <c r="O113" s="7" t="n"/>
+      <c r="P113" s="7" t="n"/>
     </row>
     <row r="114" ht="15" customHeight="1">
       <c r="A114" s="2" t="n"/>
@@ -2804,6 +3046,8 @@
       <c r="L114" s="7" t="n"/>
       <c r="M114" s="7" t="n"/>
       <c r="N114" s="3" t="n"/>
+      <c r="O114" s="7" t="n"/>
+      <c r="P114" s="7" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1">
       <c r="A115" s="2" t="n"/>
@@ -2823,6 +3067,8 @@
       <c r="L115" s="7" t="n"/>
       <c r="M115" s="7" t="n"/>
       <c r="N115" s="3" t="n"/>
+      <c r="O115" s="7" t="n"/>
+      <c r="P115" s="7" t="n"/>
     </row>
     <row r="116" ht="15" customHeight="1">
       <c r="A116" s="2" t="n"/>
@@ -2842,6 +3088,8 @@
       <c r="L116" s="7" t="n"/>
       <c r="M116" s="7" t="n"/>
       <c r="N116" s="3" t="n"/>
+      <c r="O116" s="7" t="n"/>
+      <c r="P116" s="7" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1">
       <c r="A117" s="2" t="n"/>
@@ -2861,6 +3109,8 @@
       <c r="L117" s="7" t="n"/>
       <c r="M117" s="7" t="n"/>
       <c r="N117" s="3" t="n"/>
+      <c r="O117" s="7" t="n"/>
+      <c r="P117" s="7" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1">
       <c r="A118" s="2" t="n"/>
@@ -2880,6 +3130,8 @@
       <c r="L118" s="7" t="n"/>
       <c r="M118" s="7" t="n"/>
       <c r="N118" s="3" t="n"/>
+      <c r="O118" s="7" t="n"/>
+      <c r="P118" s="7" t="n"/>
     </row>
     <row r="119" ht="15" customHeight="1">
       <c r="A119" s="2" t="n"/>
@@ -2899,6 +3151,8 @@
       <c r="L119" s="7" t="n"/>
       <c r="M119" s="7" t="n"/>
       <c r="N119" s="3" t="n"/>
+      <c r="O119" s="7" t="n"/>
+      <c r="P119" s="7" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1">
       <c r="A120" s="2" t="n"/>
@@ -2918,6 +3172,8 @@
       <c r="L120" s="7" t="n"/>
       <c r="M120" s="7" t="n"/>
       <c r="N120" s="3" t="n"/>
+      <c r="O120" s="7" t="n"/>
+      <c r="P120" s="7" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1">
       <c r="A121" s="2" t="n"/>
@@ -2937,6 +3193,8 @@
       <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="n"/>
       <c r="N121" s="3" t="n"/>
+      <c r="O121" s="7" t="n"/>
+      <c r="P121" s="7" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1">
       <c r="A122" s="2" t="n"/>
@@ -2956,6 +3214,8 @@
       <c r="L122" s="7" t="n"/>
       <c r="M122" s="7" t="n"/>
       <c r="N122" s="3" t="n"/>
+      <c r="O122" s="7" t="n"/>
+      <c r="P122" s="7" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1">
       <c r="A123" s="2" t="n"/>
@@ -2975,6 +3235,8 @@
       <c r="L123" s="7" t="n"/>
       <c r="M123" s="7" t="n"/>
       <c r="N123" s="3" t="n"/>
+      <c r="O123" s="7" t="n"/>
+      <c r="P123" s="7" t="n"/>
     </row>
     <row r="124" ht="15" customHeight="1">
       <c r="A124" s="2" t="n"/>
@@ -2994,6 +3256,8 @@
       <c r="L124" s="7" t="n"/>
       <c r="M124" s="7" t="n"/>
       <c r="N124" s="3" t="n"/>
+      <c r="O124" s="7" t="n"/>
+      <c r="P124" s="7" t="n"/>
     </row>
     <row r="125" ht="15" customHeight="1">
       <c r="A125" s="2" t="n"/>
@@ -3013,6 +3277,8 @@
       <c r="L125" s="7" t="n"/>
       <c r="M125" s="7" t="n"/>
       <c r="N125" s="3" t="n"/>
+      <c r="O125" s="7" t="n"/>
+      <c r="P125" s="7" t="n"/>
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" s="2" t="n"/>
@@ -3032,6 +3298,8 @@
       <c r="L126" s="7" t="n"/>
       <c r="M126" s="7" t="n"/>
       <c r="N126" s="3" t="n"/>
+      <c r="O126" s="7" t="n"/>
+      <c r="P126" s="7" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="A127" s="2" t="n"/>
@@ -3051,6 +3319,8 @@
       <c r="L127" s="7" t="n"/>
       <c r="M127" s="7" t="n"/>
       <c r="N127" s="3" t="n"/>
+      <c r="O127" s="7" t="n"/>
+      <c r="P127" s="7" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1">
       <c r="A128" s="2" t="n"/>
@@ -3070,6 +3340,8 @@
       <c r="L128" s="7" t="n"/>
       <c r="M128" s="7" t="n"/>
       <c r="N128" s="3" t="n"/>
+      <c r="O128" s="7" t="n"/>
+      <c r="P128" s="7" t="n"/>
     </row>
     <row r="129" ht="15" customHeight="1">
       <c r="A129" s="2" t="n"/>
@@ -3089,6 +3361,8 @@
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="3" t="n"/>
+      <c r="O129" s="7" t="n"/>
+      <c r="P129" s="7" t="n"/>
     </row>
     <row r="130" ht="15" customHeight="1">
       <c r="A130" s="2" t="n"/>
@@ -3108,6 +3382,8 @@
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="3" t="n"/>
+      <c r="O130" s="7" t="n"/>
+      <c r="P130" s="7" t="n"/>
     </row>
     <row r="131" ht="15" customHeight="1">
       <c r="A131" s="2" t="n"/>
@@ -3127,6 +3403,8 @@
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="3" t="n"/>
+      <c r="O131" s="7" t="n"/>
+      <c r="P131" s="7" t="n"/>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="A132" s="2" t="n"/>
@@ -3146,6 +3424,8 @@
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="3" t="n"/>
+      <c r="O132" s="7" t="n"/>
+      <c r="P132" s="7" t="n"/>
     </row>
     <row r="133" ht="15" customHeight="1">
       <c r="A133" s="2" t="n"/>
@@ -3165,6 +3445,8 @@
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="3" t="n"/>
+      <c r="O133" s="7" t="n"/>
+      <c r="P133" s="7" t="n"/>
     </row>
     <row r="134" ht="15" customHeight="1">
       <c r="A134" s="2" t="n"/>
@@ -3184,6 +3466,8 @@
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="3" t="n"/>
+      <c r="O134" s="7" t="n"/>
+      <c r="P134" s="7" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1">
       <c r="A135" s="2" t="n"/>
@@ -3203,6 +3487,8 @@
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="3" t="n"/>
+      <c r="O135" s="7" t="n"/>
+      <c r="P135" s="7" t="n"/>
     </row>
     <row r="136" ht="15" customHeight="1">
       <c r="A136" s="2" t="n"/>
@@ -3222,6 +3508,8 @@
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="3" t="n"/>
+      <c r="O136" s="7" t="n"/>
+      <c r="P136" s="7" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1">
       <c r="A137" s="2" t="n"/>
@@ -3241,6 +3529,8 @@
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="3" t="n"/>
+      <c r="O137" s="7" t="n"/>
+      <c r="P137" s="7" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1">
       <c r="A138" s="2" t="n"/>
@@ -3260,6 +3550,8 @@
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="3" t="n"/>
+      <c r="O138" s="7" t="n"/>
+      <c r="P138" s="7" t="n"/>
     </row>
     <row r="139" ht="15" customHeight="1">
       <c r="A139" s="2" t="n"/>
@@ -3279,6 +3571,8 @@
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="3" t="n"/>
+      <c r="O139" s="7" t="n"/>
+      <c r="P139" s="7" t="n"/>
     </row>
     <row r="140" ht="15" customHeight="1">
       <c r="A140" s="2" t="n"/>
@@ -3298,6 +3592,8 @@
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="3" t="n"/>
+      <c r="O140" s="7" t="n"/>
+      <c r="P140" s="7" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1">
       <c r="A141" s="2" t="n"/>
@@ -3317,6 +3613,8 @@
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="3" t="n"/>
+      <c r="O141" s="7" t="n"/>
+      <c r="P141" s="7" t="n"/>
     </row>
     <row r="142" ht="15" customHeight="1">
       <c r="A142" s="2" t="n"/>
@@ -3336,6 +3634,8 @@
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="3" t="n"/>
+      <c r="O142" s="7" t="n"/>
+      <c r="P142" s="7" t="n"/>
     </row>
     <row r="143" ht="15" customHeight="1">
       <c r="A143" s="2" t="n"/>
@@ -3355,6 +3655,8 @@
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="3" t="n"/>
+      <c r="O143" s="7" t="n"/>
+      <c r="P143" s="7" t="n"/>
     </row>
     <row r="144" ht="15" customHeight="1">
       <c r="A144" s="2" t="n"/>
@@ -3374,6 +3676,8 @@
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="3" t="n"/>
+      <c r="O144" s="7" t="n"/>
+      <c r="P144" s="7" t="n"/>
     </row>
     <row r="145" ht="15" customHeight="1">
       <c r="A145" s="2" t="n"/>
@@ -3393,6 +3697,8 @@
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="3" t="n"/>
+      <c r="O145" s="7" t="n"/>
+      <c r="P145" s="7" t="n"/>
     </row>
     <row r="146" ht="15" customHeight="1">
       <c r="A146" s="2" t="n"/>
@@ -3412,6 +3718,8 @@
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="3" t="n"/>
+      <c r="O146" s="7" t="n"/>
+      <c r="P146" s="7" t="n"/>
     </row>
     <row r="147" ht="15" customHeight="1">
       <c r="A147" s="2" t="n"/>
@@ -3431,6 +3739,8 @@
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="3" t="n"/>
+      <c r="O147" s="7" t="n"/>
+      <c r="P147" s="7" t="n"/>
     </row>
     <row r="148" ht="15" customHeight="1">
       <c r="A148" s="2" t="n"/>
@@ -3450,6 +3760,8 @@
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="3" t="n"/>
+      <c r="O148" s="7" t="n"/>
+      <c r="P148" s="7" t="n"/>
     </row>
     <row r="149" ht="15" customHeight="1">
       <c r="A149" s="2" t="n"/>
@@ -3469,6 +3781,8 @@
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="3" t="n"/>
+      <c r="O149" s="7" t="n"/>
+      <c r="P149" s="7" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1">
       <c r="A150" s="2" t="n"/>
@@ -3488,6 +3802,8 @@
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="3" t="n"/>
+      <c r="O150" s="7" t="n"/>
+      <c r="P150" s="7" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1">
       <c r="A151" s="2" t="n"/>
@@ -3507,6 +3823,8 @@
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="3" t="n"/>
+      <c r="O151" s="7" t="n"/>
+      <c r="P151" s="7" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1">
       <c r="A152" s="2" t="n"/>
@@ -3526,6 +3844,8 @@
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="3" t="n"/>
+      <c r="O152" s="7" t="n"/>
+      <c r="P152" s="7" t="n"/>
     </row>
     <row r="153" ht="15" customHeight="1">
       <c r="A153" s="2" t="n"/>
@@ -3545,6 +3865,8 @@
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="3" t="n"/>
+      <c r="O153" s="7" t="n"/>
+      <c r="P153" s="7" t="n"/>
     </row>
     <row r="154" ht="15" customHeight="1">
       <c r="A154" s="2" t="n"/>
@@ -3564,6 +3886,8 @@
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="3" t="n"/>
+      <c r="O154" s="7" t="n"/>
+      <c r="P154" s="7" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1">
       <c r="A155" s="2" t="n"/>
@@ -3583,6 +3907,8 @@
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="3" t="n"/>
+      <c r="O155" s="7" t="n"/>
+      <c r="P155" s="7" t="n"/>
     </row>
     <row r="156" ht="15" customHeight="1">
       <c r="A156" s="2" t="n"/>
@@ -3602,6 +3928,8 @@
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="3" t="n"/>
+      <c r="O156" s="7" t="n"/>
+      <c r="P156" s="7" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1">
       <c r="A157" s="2" t="n"/>
@@ -3621,6 +3949,8 @@
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="3" t="n"/>
+      <c r="O157" s="7" t="n"/>
+      <c r="P157" s="7" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1">
       <c r="A158" s="2" t="n"/>
@@ -3640,6 +3970,8 @@
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="3" t="n"/>
+      <c r="O158" s="7" t="n"/>
+      <c r="P158" s="7" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1">
       <c r="A159" s="2" t="n"/>
@@ -3659,6 +3991,8 @@
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="3" t="n"/>
+      <c r="O159" s="7" t="n"/>
+      <c r="P159" s="7" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1">
       <c r="A160" s="2" t="n"/>
@@ -3678,6 +4012,8 @@
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="3" t="n"/>
+      <c r="O160" s="7" t="n"/>
+      <c r="P160" s="7" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1">
       <c r="A161" s="2" t="n"/>
@@ -3697,6 +4033,8 @@
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="3" t="n"/>
+      <c r="O161" s="7" t="n"/>
+      <c r="P161" s="7" t="n"/>
     </row>
     <row r="162" ht="15" customHeight="1">
       <c r="A162" s="2" t="n"/>
@@ -3716,6 +4054,8 @@
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="3" t="n"/>
+      <c r="O162" s="7" t="n"/>
+      <c r="P162" s="7" t="n"/>
     </row>
     <row r="163" ht="15" customHeight="1">
       <c r="A163" s="2" t="n"/>
@@ -3735,6 +4075,8 @@
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="3" t="n"/>
+      <c r="O163" s="7" t="n"/>
+      <c r="P163" s="7" t="n"/>
     </row>
     <row r="164" ht="15" customHeight="1">
       <c r="A164" s="2" t="n"/>
@@ -3754,6 +4096,8 @@
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="3" t="n"/>
+      <c r="O164" s="7" t="n"/>
+      <c r="P164" s="7" t="n"/>
     </row>
     <row r="165" ht="15" customHeight="1">
       <c r="A165" s="2" t="n"/>
@@ -3773,6 +4117,8 @@
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="3" t="n"/>
+      <c r="O165" s="7" t="n"/>
+      <c r="P165" s="7" t="n"/>
     </row>
     <row r="166" ht="15" customHeight="1">
       <c r="A166" s="2" t="n"/>
@@ -3792,6 +4138,8 @@
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="3" t="n"/>
+      <c r="O166" s="7" t="n"/>
+      <c r="P166" s="7" t="n"/>
     </row>
     <row r="167" ht="15" customHeight="1">
       <c r="A167" s="2" t="n"/>
@@ -3811,6 +4159,8 @@
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="3" t="n"/>
+      <c r="O167" s="7" t="n"/>
+      <c r="P167" s="7" t="n"/>
     </row>
     <row r="168" ht="15" customHeight="1">
       <c r="A168" s="2" t="n"/>
@@ -3830,6 +4180,8 @@
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="3" t="n"/>
+      <c r="O168" s="7" t="n"/>
+      <c r="P168" s="7" t="n"/>
     </row>
     <row r="169" ht="15" customHeight="1">
       <c r="A169" s="2" t="n"/>
@@ -3849,6 +4201,8 @@
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="3" t="n"/>
+      <c r="O169" s="7" t="n"/>
+      <c r="P169" s="7" t="n"/>
     </row>
     <row r="170" ht="15" customHeight="1">
       <c r="A170" s="2" t="n"/>
@@ -3868,6 +4222,8 @@
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="3" t="n"/>
+      <c r="O170" s="7" t="n"/>
+      <c r="P170" s="7" t="n"/>
     </row>
     <row r="171" ht="15" customHeight="1">
       <c r="A171" s="2" t="n"/>
@@ -3887,6 +4243,8 @@
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="3" t="n"/>
+      <c r="O171" s="7" t="n"/>
+      <c r="P171" s="7" t="n"/>
     </row>
     <row r="172" ht="15" customHeight="1">
       <c r="A172" s="2" t="n"/>
@@ -3906,6 +4264,8 @@
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="3" t="n"/>
+      <c r="O172" s="7" t="n"/>
+      <c r="P172" s="7" t="n"/>
     </row>
     <row r="173" ht="15" customHeight="1">
       <c r="A173" s="2" t="n"/>
@@ -3925,6 +4285,8 @@
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="3" t="n"/>
+      <c r="O173" s="7" t="n"/>
+      <c r="P173" s="7" t="n"/>
     </row>
     <row r="174" ht="15" customHeight="1">
       <c r="A174" s="2" t="n"/>
@@ -3944,6 +4306,8 @@
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="3" t="n"/>
+      <c r="O174" s="7" t="n"/>
+      <c r="P174" s="7" t="n"/>
     </row>
     <row r="175" ht="15" customHeight="1">
       <c r="A175" s="2" t="n"/>
@@ -3963,6 +4327,8 @@
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="3" t="n"/>
+      <c r="O175" s="7" t="n"/>
+      <c r="P175" s="7" t="n"/>
     </row>
     <row r="176" ht="15" customHeight="1">
       <c r="A176" s="2" t="n"/>
@@ -3982,6 +4348,8 @@
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
       <c r="N176" s="3" t="n"/>
+      <c r="O176" s="7" t="n"/>
+      <c r="P176" s="7" t="n"/>
     </row>
     <row r="177" ht="15" customHeight="1">
       <c r="A177" s="2" t="n"/>
@@ -4001,6 +4369,8 @@
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="3" t="n"/>
+      <c r="O177" s="7" t="n"/>
+      <c r="P177" s="7" t="n"/>
     </row>
     <row r="178" ht="15" customHeight="1">
       <c r="A178" s="2" t="n"/>
@@ -4020,6 +4390,8 @@
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="3" t="n"/>
+      <c r="O178" s="7" t="n"/>
+      <c r="P178" s="7" t="n"/>
     </row>
     <row r="179" ht="15" customHeight="1">
       <c r="A179" s="2" t="n"/>
@@ -4039,6 +4411,8 @@
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="3" t="n"/>
+      <c r="O179" s="7" t="n"/>
+      <c r="P179" s="7" t="n"/>
     </row>
     <row r="180" ht="15" customHeight="1">
       <c r="A180" s="2" t="n"/>
@@ -4058,6 +4432,8 @@
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="3" t="n"/>
+      <c r="O180" s="7" t="n"/>
+      <c r="P180" s="7" t="n"/>
     </row>
     <row r="181" ht="15" customHeight="1">
       <c r="A181" s="2" t="n"/>
@@ -4077,6 +4453,8 @@
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="3" t="n"/>
+      <c r="O181" s="7" t="n"/>
+      <c r="P181" s="7" t="n"/>
     </row>
     <row r="182" ht="15" customHeight="1">
       <c r="A182" s="2" t="n"/>
@@ -4096,6 +4474,8 @@
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="3" t="n"/>
+      <c r="O182" s="7" t="n"/>
+      <c r="P182" s="7" t="n"/>
     </row>
     <row r="183" ht="15" customHeight="1">
       <c r="A183" s="2" t="n"/>
@@ -4115,6 +4495,8 @@
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="3" t="n"/>
+      <c r="O183" s="7" t="n"/>
+      <c r="P183" s="7" t="n"/>
     </row>
     <row r="184" ht="15" customHeight="1">
       <c r="A184" s="2" t="n"/>
@@ -4134,6 +4516,8 @@
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="3" t="n"/>
+      <c r="O184" s="7" t="n"/>
+      <c r="P184" s="7" t="n"/>
     </row>
     <row r="185" ht="15" customHeight="1">
       <c r="A185" s="2" t="n"/>
@@ -4153,6 +4537,8 @@
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="3" t="n"/>
+      <c r="O185" s="7" t="n"/>
+      <c r="P185" s="7" t="n"/>
     </row>
     <row r="186" ht="15" customHeight="1">
       <c r="A186" s="2" t="n"/>
@@ -4172,6 +4558,8 @@
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="3" t="n"/>
+      <c r="O186" s="7" t="n"/>
+      <c r="P186" s="7" t="n"/>
     </row>
     <row r="187" ht="15" customHeight="1">
       <c r="A187" s="2" t="n"/>
@@ -4191,6 +4579,8 @@
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="3" t="n"/>
+      <c r="O187" s="7" t="n"/>
+      <c r="P187" s="7" t="n"/>
     </row>
     <row r="188" ht="15" customHeight="1">
       <c r="A188" s="2" t="n"/>
@@ -4210,6 +4600,8 @@
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="3" t="n"/>
+      <c r="O188" s="7" t="n"/>
+      <c r="P188" s="7" t="n"/>
     </row>
     <row r="189" ht="15" customHeight="1">
       <c r="A189" s="2" t="n"/>
@@ -4229,6 +4621,8 @@
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="3" t="n"/>
+      <c r="O189" s="7" t="n"/>
+      <c r="P189" s="7" t="n"/>
     </row>
     <row r="190" ht="15" customHeight="1">
       <c r="A190" s="2" t="n"/>
@@ -4248,6 +4642,8 @@
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="3" t="n"/>
+      <c r="O190" s="7" t="n"/>
+      <c r="P190" s="7" t="n"/>
     </row>
     <row r="191" ht="15" customHeight="1">
       <c r="A191" s="2" t="n"/>
@@ -4267,6 +4663,8 @@
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="3" t="n"/>
+      <c r="O191" s="7" t="n"/>
+      <c r="P191" s="7" t="n"/>
     </row>
     <row r="192" ht="15" customHeight="1">
       <c r="A192" s="2" t="n"/>
@@ -4286,6 +4684,8 @@
       <c r="L192" s="7" t="n"/>
       <c r="M192" s="7" t="n"/>
       <c r="N192" s="3" t="n"/>
+      <c r="O192" s="7" t="n"/>
+      <c r="P192" s="7" t="n"/>
     </row>
     <row r="193" ht="15" customHeight="1">
       <c r="A193" s="2" t="n"/>
@@ -4305,6 +4705,8 @@
       <c r="L193" s="7" t="n"/>
       <c r="M193" s="7" t="n"/>
       <c r="N193" s="3" t="n"/>
+      <c r="O193" s="7" t="n"/>
+      <c r="P193" s="7" t="n"/>
     </row>
     <row r="194" ht="15" customHeight="1">
       <c r="A194" s="2" t="n"/>
@@ -4324,6 +4726,8 @@
       <c r="L194" s="7" t="n"/>
       <c r="M194" s="7" t="n"/>
       <c r="N194" s="3" t="n"/>
+      <c r="O194" s="7" t="n"/>
+      <c r="P194" s="7" t="n"/>
     </row>
     <row r="195" ht="15" customHeight="1">
       <c r="A195" s="2" t="n"/>
@@ -4343,6 +4747,8 @@
       <c r="L195" s="7" t="n"/>
       <c r="M195" s="7" t="n"/>
       <c r="N195" s="3" t="n"/>
+      <c r="O195" s="7" t="n"/>
+      <c r="P195" s="7" t="n"/>
     </row>
     <row r="196" ht="15" customHeight="1">
       <c r="A196" s="2" t="n"/>
@@ -4362,6 +4768,8 @@
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="3" t="n"/>
+      <c r="O196" s="7" t="n"/>
+      <c r="P196" s="7" t="n"/>
     </row>
     <row r="197" ht="15" customHeight="1">
       <c r="A197" s="2" t="n"/>
@@ -4381,6 +4789,8 @@
       <c r="L197" s="7" t="n"/>
       <c r="M197" s="7" t="n"/>
       <c r="N197" s="3" t="n"/>
+      <c r="O197" s="7" t="n"/>
+      <c r="P197" s="7" t="n"/>
     </row>
     <row r="198" ht="15" customHeight="1">
       <c r="A198" s="2" t="n"/>
@@ -4400,6 +4810,8 @@
       <c r="L198" s="7" t="n"/>
       <c r="M198" s="7" t="n"/>
       <c r="N198" s="3" t="n"/>
+      <c r="O198" s="7" t="n"/>
+      <c r="P198" s="7" t="n"/>
     </row>
     <row r="199" ht="15" customHeight="1">
       <c r="A199" s="2" t="n"/>
@@ -4419,6 +4831,8 @@
       <c r="L199" s="7" t="n"/>
       <c r="M199" s="7" t="n"/>
       <c r="N199" s="3" t="n"/>
+      <c r="O199" s="7" t="n"/>
+      <c r="P199" s="7" t="n"/>
     </row>
     <row r="200" ht="15" customHeight="1">
       <c r="A200" s="2" t="n"/>
@@ -4438,6 +4852,8 @@
       <c r="L200" s="7" t="n"/>
       <c r="M200" s="7" t="n"/>
       <c r="N200" s="3" t="n"/>
+      <c r="O200" s="7" t="n"/>
+      <c r="P200" s="7" t="n"/>
     </row>
     <row r="201" ht="15" customHeight="1">
       <c r="A201" s="2" t="n"/>
@@ -4457,11 +4873,13 @@
       <c r="L201" s="7" t="n"/>
       <c r="M201" s="7" t="n"/>
       <c r="N201" s="3" t="n"/>
+      <c r="O201" s="7" t="n"/>
+      <c r="P201" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="A2:A201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"neu,fertig,Fehler"</formula1>
+      <formula1>"neu,fertig,Fehler,abgelaufen"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4469,7 +4887,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="N2:N201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Technik,Haushalt,Küche,Sport &amp; Freizeit,Beauty &amp; Pflege,Spielzeug,Garten &amp; Baumarkt,Sonstiges"</formula1>
+      <formula1>"Technik,Gaming,Haushalt,Küche,Mode,Beauty &amp; Pflege,Sport &amp; Freizeit,Spielzeug,Baby &amp; Kind,Garten &amp; Baumarkt,Tierbedarf,Sonstiges"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Neuer Deal #2: Amazon-Produkt B0GJD7VMPX
</commit_message>
<xml_diff>
--- a/deals.xlsx
+++ b/deals.xlsx
@@ -740,25 +740,67 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>amazon-produkt-b0gjd7vmpx</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Amazon-Produkt B0GJD7VMPX</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>664</v>
+      </c>
       <c r="F5" s="5">
         <f>IF(AND(ISNUMBER(D5),ISNUMBER(E5),D5&gt;E5),1-E5/D5,"")</f>
         <v/>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>25.10.2026, 17:28</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.de/dp/B0GJD7VMPX</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>DEAL</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
       <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>B0GJD7VMPX</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="n"/>

</xml_diff>